<commit_message>
Fix generated catalog asset paths
</commit_message>
<xml_diff>
--- a/data/import/alcantara/alcantara.xlsx
+++ b/data/import/alcantara/alcantara.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="900" windowWidth="34200" windowHeight="19720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="product_types" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="product_type_specs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="product_type_certifications" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="product_type_maintenance" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="skus" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sku_specs" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="product_type_downloads" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sku_case_gallery" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="product_types" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="product_type_specs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="product_type_certifications" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="product_type_maintenance" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="skus" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="sku_specs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="product_type_downloads" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="sku_case_gallery" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'product_types'!$A$1:$I$3</definedName>
@@ -732,7 +732,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>/public/uploads/alcantara/panel/alcantara-panel-hero.jpg</t>
+          <t>/uploads/alcantara/panel/1108.jpg</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -794,11 +794,13 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>/public/uploads/alcantara/cover/alcantara-cover-hero.jpg</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="n">
-        <v>5205</v>
+          <t>/uploads/alcantara/panel/1108.jpg</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>5205</t>
+        </is>
       </c>
     </row>
     <row r="4" ht="75" customHeight="1">
@@ -40023,7 +40025,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>/uploads/spec/Alcantara 5012 - Pannel.pdf</t>
+          <t>/uploads/spec/Alcantara/Alcantara 5012 - Pannel.pdf</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -40063,7 +40065,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>/uploads/spec/Instructions-for-maintenance-of-alcantara-material.pdf</t>
+          <t>/uploads/spec/Alcantara/Instructions-for-maintenance-of-alcantara-material.pdf</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -40103,7 +40105,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>/uploads/spec/Alcantara 5205 - COVER Spec sheet.pdf</t>
+          <t>/uploads/spec/Alcantara/Alcantara 5205 - COVER Spec sheet.pdf</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -40143,7 +40145,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>/uploads/spec/Instructions-for-maintenance-of-alcantara-material.pdf</t>
+          <t>/uploads/spec/Alcantara/Instructions-for-maintenance-of-alcantara-material.pdf</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -40183,7 +40185,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>/uploads/spec/Alcantara 5015 ( BP ) Regular.pdf</t>
+          <t>/uploads/spec/Alcantara/Alcantara 5015 ( BP ) Regular.pdf</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -40223,7 +40225,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>/uploads/spec/Instructions-for-maintenance-of-alcantara-material.pdf</t>
+          <t>/uploads/spec/Alcantara/Instructions-for-maintenance-of-alcantara-material.pdf</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -40263,7 +40265,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>/uploads/spec/Alcantara 5143 - EXO.pdf</t>
+          <t>/uploads/spec/Alcantara/Alcantara 5143 - EXO.pdf</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -40303,7 +40305,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>/uploads/spec/Instructions-for-maintenance-of-alcantara-material.pdf</t>
+          <t>/uploads/spec/Alcantara/Instructions-for-maintenance-of-alcantara-material.pdf</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -40343,7 +40345,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>/uploads/spec/Alcantara 5010 - 0.4 Thin 5010 Datasheet(1).pdf</t>
+          <t>/uploads/spec/Alcantara/Alcantara 5010 - 0.4 Thin 5010 Datasheet(1).pdf</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -40383,7 +40385,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>/uploads/spec/Alcantara 5030 - 0.4 Thin ECG.pdf</t>
+          <t>/uploads/spec/Alcantara/Alcantara 5030 - 0.4 Thin ECG.pdf</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -40423,7 +40425,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>/uploads/spec/Instructions-for-maintenance-of-alcantara-material.pdf</t>
+          <t>/uploads/spec/Alcantara/Instructions-for-maintenance-of-alcantara-material.pdf</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -40463,7 +40465,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>/uploads/spec/Alcantara 5170 Multilayer.pdf</t>
+          <t>/uploads/spec/Alcantara/Alcantara 5170 Multilayer.pdf</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -40503,7 +40505,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>/uploads/spec/Instructions-for-maintenance-of-alcantara-material.pdf</t>
+          <t>/uploads/spec/Alcantara/Instructions-for-maintenance-of-alcantara-material.pdf</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -40543,7 +40545,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>/uploads/spec/Alcantara 5466 - Avant.pdf</t>
+          <t>/uploads/spec/Alcantara/Alcantara 5466 - Avant.pdf</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -40583,7 +40585,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>/uploads/spec/Instructions-for-maintenance-of-alcantara-material.pdf</t>
+          <t>/uploads/spec/Alcantara/Instructions-for-maintenance-of-alcantara-material.pdf</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -40623,7 +40625,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>/uploads/spec/Alcantara Bord FR 5056.pdf</t>
+          <t>/uploads/spec/Alcantara/Alcantara Bord FR 5056.pdf</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -40663,7 +40665,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>/uploads/spec/Instructions-for-maintenance-of-alcantara-material.pdf</t>
+          <t>/uploads/spec/Alcantara/Instructions-for-maintenance-of-alcantara-material.pdf</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">

</xml_diff>